<commit_message>
Updated Test Log with git hashes
</commit_message>
<xml_diff>
--- a/Test_Log.xlsx
+++ b/Test_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Games Programming\GAMR2541\LabWork\angry-birds-clone-assignment-NE12follow1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A22361-A5C6-48A2-8225-A28FABF87259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDAAA23-3CBE-4E16-A146-E3D5C79AB1BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
   </bookViews>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="40">
   <si>
     <t>Date:</t>
   </si>
@@ -306,6 +306,9 @@
   </si>
   <si>
     <t>enemy set function for type works</t>
+  </si>
+  <si>
+    <t>17330a6</t>
   </si>
 </sst>
 </file>
@@ -1154,7 +1157,9 @@
       <c r="B9" s="3">
         <v>46135</v>
       </c>
-      <c r="C9" s="9"/>
+      <c r="C9" s="9" t="s">
+        <v>39</v>
+      </c>
       <c r="D9" s="6" t="s">
         <v>32</v>
       </c>
@@ -1182,7 +1187,9 @@
       <c r="B10" s="3">
         <v>46135</v>
       </c>
-      <c r="C10" s="9"/>
+      <c r="C10" s="9" t="s">
+        <v>39</v>
+      </c>
       <c r="D10" s="6" t="s">
         <v>35</v>
       </c>
@@ -1210,7 +1217,9 @@
       <c r="B11" s="3">
         <v>46135</v>
       </c>
-      <c r="C11" s="9"/>
+      <c r="C11" s="9" t="s">
+        <v>39</v>
+      </c>
       <c r="D11" s="6" t="s">
         <v>36</v>
       </c>

</xml_diff>